<commit_message>
Con extracción de fechas vigencia  y ingreso al SII
</commit_message>
<xml_diff>
--- a/Configuracion/Config.xlsx
+++ b/Configuracion/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\uipath\RIBA24GMXcmx01_Endosos\Configuracion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17186895-8937-447B-9671-57BF0D0E95FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72223CE0-66FA-4572-9320-BC5BB524B294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16615" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16615" uniqueCount="217">
   <si>
     <t>Nombre</t>
   </si>
@@ -686,6 +686,9 @@
   <si>
     <t>https://panel-rpa-servicios.optimus-799.workers.dev</t>
   </si>
+  <si>
+    <t xml:space="preserve">N </t>
+  </si>
 </sst>
 </file>
 
@@ -52425,7 +52428,7 @@
         <v>108</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>145</v>
+        <v>216</v>
       </c>
     </row>
     <row r="115" spans="1:26" x14ac:dyDescent="0.25">

</xml_diff>